<commit_message>
Multiple UI & Email Notification related changes
</commit_message>
<xml_diff>
--- a/public/Actimize_SSB1_template.xlsx
+++ b/public/Actimize_SSB1_template.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Template" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference Values" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,23 +425,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:X4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="33" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="23" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="33" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="19" customWidth="1" min="23" max="23"/>
+    <col width="43" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,60 +467,110 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>CustomerType</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>PrimaryFirstName</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>PrimaryMiddleName</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PrimaryLastName</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PrimaryFullName</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Alias1FullName</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>DateOfBirth</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Address1Line1</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Address1Line2</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Address1City</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Address1StateProvince</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Address1ZipCode</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Address1Country</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>CountryOfBirth</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>NationalityCountry1</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Countries</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Addresses</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>PartyId1Type</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>PartyId1Value</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>PartyId1IDCountry</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -530,56 +589,106 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>John</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Smith</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
         <is>
           <t>Johnny Smith</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>1980-01-15</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>123 Main St</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Apt 5</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>10001</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>123 Main St, New York, NY 10001</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
         <is>
           <t>PASSPORT</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>P1234567</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>Individual sample (PartyType I)</t>
         </is>
@@ -596,42 +705,80 @@
           <t>E</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>Prudential Asset Management LLC</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Prudential AM</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>751 Broad St</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Newark</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>07102</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>751 Broad St, Newark, NJ 07102</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
         <is>
           <t>REGISTRATION</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>REG-998877</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>Organization sample (PartyType E)</t>
         </is>
@@ -648,182 +795,78 @@
           <t>X</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Entity</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Unknown Counterparty Example</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Unknown CP</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>10 Bishopsgate</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>EC2N 4BQ</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>10 Bishopsgate, London EC2N 4BQ</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
         <is>
           <t>TIN</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>TIN-4455</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Unknown sample (any PartyType other than I/E)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Allowed Value</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>PartyType</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Individual</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>PartyType</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>PartyType</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Other character</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Gender</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>(blank)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Unknown</t>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Unknown sample (PartyType other than I/E)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove Wrong key from template
</commit_message>
<xml_diff>
--- a/public/Actimize_SSB1_template.xlsx
+++ b/public/Actimize_SSB1_template.xlsx
@@ -397,267 +397,263 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BK1"/>
+  <dimension ref="A1:BJ1"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="19.83203125" customWidth="1"/>
-    <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="19.83203125" customWidth="1"/>
-    <col min="10" max="10" width="14.83203125" customWidth="1"/>
-    <col min="11" max="11" width="15.83203125" customWidth="1"/>
-    <col min="12" max="12" width="19.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" customWidth="1"/>
-    <col min="15" max="15" width="17.83203125" customWidth="1"/>
-    <col min="16" max="16" width="19.83203125" customWidth="1"/>
-    <col min="17" max="17" width="17.83203125" customWidth="1"/>
-    <col min="18" max="18" width="21.83203125" customWidth="1"/>
-    <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="18.83203125" customWidth="1"/>
-    <col min="21" max="21" width="16.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.83203125" customWidth="1"/>
-    <col min="23" max="23" width="16.83203125" customWidth="1"/>
-    <col min="24" max="24" width="20.83203125" customWidth="1"/>
-    <col min="25" max="25" width="17.83203125" customWidth="1"/>
-    <col min="26" max="26" width="18.83203125" customWidth="1"/>
-    <col min="27" max="27" width="16.83203125" customWidth="1"/>
-    <col min="28" max="28" width="18.83203125" customWidth="1"/>
-    <col min="29" max="29" width="16.83203125" customWidth="1"/>
-    <col min="30" max="30" width="20.83203125" customWidth="1"/>
-    <col min="31" max="31" width="17.83203125" customWidth="1"/>
-    <col min="32" max="32" width="18.83203125" customWidth="1"/>
-    <col min="33" max="33" width="16.83203125" customWidth="1"/>
-    <col min="34" max="34" width="18.83203125" customWidth="1"/>
-    <col min="35" max="35" width="16.83203125" customWidth="1"/>
-    <col min="36" max="36" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="19.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="19.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" customWidth="1"/>
+    <col min="11" max="11" width="19.83203125" customWidth="1"/>
+    <col min="12" max="12" width="18.83203125" customWidth="1"/>
+    <col min="13" max="13" width="19.83203125" customWidth="1"/>
+    <col min="14" max="14" width="17.83203125" customWidth="1"/>
+    <col min="15" max="15" width="19.83203125" customWidth="1"/>
+    <col min="16" max="16" width="17.83203125" customWidth="1"/>
+    <col min="17" max="17" width="21.83203125" customWidth="1"/>
+    <col min="18" max="18" width="17.83203125" customWidth="1"/>
+    <col min="19" max="19" width="18.83203125" customWidth="1"/>
+    <col min="20" max="20" width="16.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="16.83203125" customWidth="1"/>
+    <col min="23" max="23" width="20.83203125" customWidth="1"/>
+    <col min="24" max="24" width="17.83203125" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" customWidth="1"/>
+    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="28" max="28" width="16.83203125" customWidth="1"/>
+    <col min="29" max="29" width="20.83203125" customWidth="1"/>
+    <col min="30" max="30" width="17.83203125" customWidth="1"/>
+    <col min="31" max="31" width="18.83203125" customWidth="1"/>
+    <col min="32" max="32" width="16.83203125" customWidth="1"/>
+    <col min="33" max="33" width="18.83203125" customWidth="1"/>
+    <col min="34" max="34" width="16.83203125" customWidth="1"/>
+    <col min="35" max="35" width="20.83203125" customWidth="1"/>
+    <col min="36" max="36" width="15.83203125" customWidth="1"/>
     <col min="37" max="37" width="15.83203125" customWidth="1"/>
-    <col min="38" max="38" width="15.83203125" customWidth="1"/>
-    <col min="39" max="39" width="14.83203125" customWidth="1"/>
+    <col min="38" max="38" width="14.83203125" customWidth="1"/>
+    <col min="39" max="39" width="17.83203125" customWidth="1"/>
     <col min="40" max="40" width="17.83203125" customWidth="1"/>
-    <col min="41" max="41" width="17.83203125" customWidth="1"/>
-    <col min="42" max="42" width="23.83203125" customWidth="1"/>
+    <col min="41" max="41" width="23.83203125" customWidth="1"/>
+    <col min="42" max="42" width="15.83203125" customWidth="1"/>
     <col min="43" max="43" width="15.83203125" customWidth="1"/>
-    <col min="44" max="44" width="15.83203125" customWidth="1"/>
-    <col min="45" max="45" width="14.83203125" customWidth="1"/>
+    <col min="44" max="44" width="14.83203125" customWidth="1"/>
+    <col min="45" max="45" width="17.83203125" customWidth="1"/>
     <col min="46" max="46" width="17.83203125" customWidth="1"/>
-    <col min="47" max="47" width="17.83203125" customWidth="1"/>
-    <col min="48" max="48" width="23.83203125" customWidth="1"/>
+    <col min="47" max="47" width="23.83203125" customWidth="1"/>
+    <col min="48" max="48" width="15.83203125" customWidth="1"/>
     <col min="49" max="49" width="15.83203125" customWidth="1"/>
-    <col min="50" max="50" width="15.83203125" customWidth="1"/>
-    <col min="51" max="51" width="14.83203125" customWidth="1"/>
+    <col min="50" max="50" width="14.83203125" customWidth="1"/>
+    <col min="51" max="51" width="17.83203125" customWidth="1"/>
     <col min="52" max="52" width="17.83203125" customWidth="1"/>
-    <col min="53" max="53" width="17.83203125" customWidth="1"/>
-    <col min="54" max="54" width="23.83203125" customWidth="1"/>
+    <col min="53" max="53" width="23.83203125" customWidth="1"/>
+    <col min="54" max="54" width="14.83203125" customWidth="1"/>
     <col min="55" max="55" width="14.83203125" customWidth="1"/>
     <col min="56" max="56" width="14.83203125" customWidth="1"/>
-    <col min="57" max="57" width="14.83203125" customWidth="1"/>
-    <col min="58" max="58" width="15.83203125" customWidth="1"/>
+    <col min="57" max="57" width="15.83203125" customWidth="1"/>
+    <col min="58" max="58" width="21.83203125" customWidth="1"/>
     <col min="59" max="59" width="21.83203125" customWidth="1"/>
     <col min="60" max="60" width="21.83203125" customWidth="1"/>
-    <col min="61" max="61" width="21.83203125" customWidth="1"/>
+    <col min="61" max="61" width="14.83203125" customWidth="1"/>
     <col min="62" max="62" width="14.83203125" customWidth="1"/>
-    <col min="63" max="63" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Attribute</v>
+        <v>PartyKey</v>
       </c>
       <c r="B1" t="str">
-        <v>PartyKey</v>
+        <v>PartyType</v>
       </c>
       <c r="C1" t="str">
-        <v>PartyType</v>
+        <v>PartyId1Type</v>
       </c>
       <c r="D1" t="str">
-        <v>PartyId1Type</v>
+        <v>PartyId1Value</v>
       </c>
       <c r="E1" t="str">
-        <v>PartyId1Value</v>
+        <v>PartyId1IDCountry</v>
       </c>
       <c r="F1" t="str">
-        <v>PartyId1IDCountry</v>
+        <v>PartyId2Type</v>
       </c>
       <c r="G1" t="str">
-        <v>PartyId2Type</v>
+        <v>PartyId2Value</v>
       </c>
       <c r="H1" t="str">
-        <v>PartyId2Value</v>
+        <v>PartyId2IDCountry</v>
       </c>
       <c r="I1" t="str">
-        <v>PartyId2IDCountry</v>
+        <v>PartyId3Type</v>
       </c>
       <c r="J1" t="str">
-        <v>PartyId3Type</v>
+        <v>PartyId3Value</v>
       </c>
       <c r="K1" t="str">
-        <v>PartyId3Value</v>
+        <v>PartyId3IDCountry</v>
       </c>
       <c r="L1" t="str">
-        <v>PartyId3IDCountry</v>
+        <v>PrimaryFirstName</v>
       </c>
       <c r="M1" t="str">
-        <v>PrimaryFirstName</v>
+        <v>PrimaryMiddleName</v>
       </c>
       <c r="N1" t="str">
-        <v>PrimaryMiddleName</v>
+        <v>PrimaryLastName</v>
       </c>
       <c r="O1" t="str">
-        <v>PrimaryLastName</v>
+        <v>PrimaryMaidenName</v>
       </c>
       <c r="P1" t="str">
-        <v>PrimaryMaidenName</v>
+        <v>PrimaryFullName</v>
       </c>
       <c r="Q1" t="str">
-        <v>PrimaryFullName</v>
+        <v>PrimaryIsBrokenName</v>
       </c>
       <c r="R1" t="str">
-        <v>PrimaryIsBrokenName</v>
+        <v>Alias1FirstName</v>
       </c>
       <c r="S1" t="str">
-        <v>Alias1FirstName</v>
+        <v>Alias1MiddleName</v>
       </c>
       <c r="T1" t="str">
-        <v>Alias1MiddleName</v>
+        <v>Alias1LastName</v>
       </c>
       <c r="U1" t="str">
-        <v>Alias1LastName</v>
+        <v>Alias1MaidenName</v>
       </c>
       <c r="V1" t="str">
-        <v>Alias1MaidenName</v>
+        <v>Alias1FullName</v>
       </c>
       <c r="W1" t="str">
-        <v>Alias1FullName</v>
+        <v>Alias1IsBrokenName</v>
       </c>
       <c r="X1" t="str">
-        <v>Alias1IsBrokenName</v>
+        <v>Alias2FirstName</v>
       </c>
       <c r="Y1" t="str">
-        <v>Alias2FirstName</v>
+        <v>Alias2MiddleName</v>
       </c>
       <c r="Z1" t="str">
-        <v>Alias2MiddleName</v>
+        <v>Alias2LastName</v>
       </c>
       <c r="AA1" t="str">
-        <v>Alias2LastName</v>
+        <v>Alias2MaidenName</v>
       </c>
       <c r="AB1" t="str">
-        <v>Alias2MaidenName</v>
+        <v>Alias2FullName</v>
       </c>
       <c r="AC1" t="str">
-        <v>Alias2FullName</v>
+        <v>Alias2IsBrokenName</v>
       </c>
       <c r="AD1" t="str">
-        <v>Alias2IsBrokenName</v>
+        <v>Alias3FirstName</v>
       </c>
       <c r="AE1" t="str">
-        <v>Alias3FirstName</v>
+        <v>Alias3MiddleName</v>
       </c>
       <c r="AF1" t="str">
-        <v>Alias3MiddleName</v>
+        <v>Alias3LastName</v>
       </c>
       <c r="AG1" t="str">
-        <v>Alias3LastName</v>
+        <v>Alias3MaidenName</v>
       </c>
       <c r="AH1" t="str">
-        <v>Alias3MaidenName</v>
+        <v>Alias3FullName</v>
       </c>
       <c r="AI1" t="str">
-        <v>Alias3FullName</v>
+        <v>Alias3IsBrokenName</v>
       </c>
       <c r="AJ1" t="str">
-        <v>Alias3IsBrokenName</v>
+        <v>Address1Line1</v>
       </c>
       <c r="AK1" t="str">
-        <v>Address1Line1</v>
+        <v>Address1Line2</v>
       </c>
       <c r="AL1" t="str">
-        <v>Address1Line2</v>
+        <v>Address1City</v>
       </c>
       <c r="AM1" t="str">
-        <v>Address1City</v>
+        <v>Address1ZipCode</v>
       </c>
       <c r="AN1" t="str">
-        <v>Address1ZipCode</v>
+        <v>Address1Country</v>
       </c>
       <c r="AO1" t="str">
-        <v>Address1Country</v>
+        <v>Address1stateProvince</v>
       </c>
       <c r="AP1" t="str">
-        <v>Address1stateProvince</v>
+        <v>Address2Line1</v>
       </c>
       <c r="AQ1" t="str">
-        <v>Address2Line1</v>
+        <v>Address2Line2</v>
       </c>
       <c r="AR1" t="str">
-        <v>Address2Line2</v>
+        <v>Address2City</v>
       </c>
       <c r="AS1" t="str">
-        <v>Address2City</v>
+        <v>Address2ZipCode</v>
       </c>
       <c r="AT1" t="str">
-        <v>Address2ZipCode</v>
+        <v>Address2Country</v>
       </c>
       <c r="AU1" t="str">
-        <v>Address2Country</v>
+        <v>Address2stateProvince</v>
       </c>
       <c r="AV1" t="str">
-        <v>Address2stateProvince</v>
+        <v>Address3Line1</v>
       </c>
       <c r="AW1" t="str">
-        <v>Address3Line1</v>
+        <v>Address3Line2</v>
       </c>
       <c r="AX1" t="str">
-        <v>Address3Line2</v>
+        <v>Address3City</v>
       </c>
       <c r="AY1" t="str">
-        <v>Address3City</v>
+        <v>Address3ZipCode</v>
       </c>
       <c r="AZ1" t="str">
-        <v>Address3ZipCode</v>
+        <v>Address3Country</v>
       </c>
       <c r="BA1" t="str">
-        <v>Address3Country</v>
+        <v>Address3stateProvince</v>
       </c>
       <c r="BB1" t="str">
-        <v>Address3stateProvince</v>
+        <v>DateOfBirth</v>
       </c>
       <c r="BC1" t="str">
-        <v>DateOfBirth</v>
+        <v>YearOfBirth</v>
       </c>
       <c r="BD1" t="str">
-        <v>YearOfBirth</v>
+        <v>BirthCountry</v>
       </c>
       <c r="BE1" t="str">
-        <v>BirthCountry</v>
+        <v>BirthLocation</v>
       </c>
       <c r="BF1" t="str">
-        <v>BirthLocation</v>
+        <v>NationalityCountry1</v>
       </c>
       <c r="BG1" t="str">
-        <v>NationalityCountry1</v>
+        <v>NationalityCountry2</v>
       </c>
       <c r="BH1" t="str">
-        <v>NationalityCountry2</v>
+        <v>NationalityCountry3</v>
       </c>
       <c r="BI1" t="str">
-        <v>NationalityCountry3</v>
+        <v>Gender</v>
       </c>
       <c r="BJ1" t="str">
-        <v>Gender</v>
-      </c>
-      <c r="BK1" t="str">
         <v>Title</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BK1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BJ1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change retry  to 5 times and adding A04 :400 error as retry mechanism
</commit_message>
<xml_diff>
--- a/public/Actimize_SSB1_template.xlsx
+++ b/public/Actimize_SSB1_template.xlsx
@@ -678,7 +678,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>7. Country fields (Address*, BirthCountry, NationalityCountry*) must use ISO 3166-1 alpha-2 codes (example: US, IN, GB).</t>
+          <t>7. Country fields (Address*, BirthCountry, NationalityCountry*) must use ISO 3166-1 alpha-3 codes (example: USA, IND, GBR).</t>
         </is>
       </c>
       <c r="B11" s="9" t="n"/>
@@ -783,7 +783,7 @@
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>ISO alpha-2 uppercase</t>
+          <t>ISO alpha-3 uppercase</t>
         </is>
       </c>
       <c r="C21" s="12" t="inlineStr">
@@ -886,8 +886,8 @@
   <mergeCells count="4">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A27:C27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2130,12 +2130,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="C66:C67"/>
+    <mergeCell ref="B66:B67"/>
+    <mergeCell ref="C3:C7"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C3:C7"/>
     <mergeCell ref="A66:A67"/>
-    <mergeCell ref="B66:B67"/>
-    <mergeCell ref="C66:C67"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="F2" s="12" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="H2" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="I2" s="12" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="K2" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="L2" s="12" t="inlineStr">
@@ -2724,7 +2724,7 @@
       </c>
       <c r="AN2" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="AO2" s="12" t="inlineStr">
@@ -2754,7 +2754,7 @@
       </c>
       <c r="AT2" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="AU2" s="12" t="inlineStr">
@@ -2784,7 +2784,7 @@
       </c>
       <c r="AZ2" s="12" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="BA2" s="12" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="BD2" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="BE2" s="12" t="inlineStr">
@@ -2814,17 +2814,17 @@
       </c>
       <c r="BF2" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="BG2" s="12" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="BH2" s="12" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>GBR</t>
         </is>
       </c>
       <c r="BI2" s="12" t="inlineStr">
@@ -2861,159 +2861,159 @@
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>PASSPORT</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>E99887766</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>GBR</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>SSN</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>999-11-2222</t>
+        </is>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>Acme</t>
+        </is>
+      </c>
+      <c r="M3" s="12" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="N3" s="12" t="inlineStr">
+        <is>
+          <t>Holdings</t>
+        </is>
+      </c>
+      <c r="O3" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="P3" s="12" t="inlineStr">
+        <is>
+          <t>Acme Global Holdings LLC</t>
+        </is>
+      </c>
+      <c r="Q3" s="12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="R3" s="12" t="inlineStr">
+        <is>
+          <t>Acme</t>
+        </is>
+      </c>
+      <c r="S3" s="12" t="inlineStr">
+        <is>
+          <t>Intl</t>
+        </is>
+      </c>
+      <c r="T3" s="12" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="U3" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="V3" s="12" t="inlineStr">
+        <is>
+          <t>Acme International Group</t>
+        </is>
+      </c>
+      <c r="W3" s="12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="X3" s="12" t="inlineStr">
+        <is>
+          <t>AGH</t>
+        </is>
+      </c>
+      <c r="Y3" s="12" t="inlineStr">
+        <is>
+          <t>Corp</t>
+        </is>
+      </c>
+      <c r="Z3" s="12" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>PASSPORT</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>E99887766</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>SSN</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="inlineStr">
-        <is>
-          <t>999-11-2222</t>
-        </is>
-      </c>
-      <c r="K3" s="12" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="L3" s="12" t="inlineStr">
+      <c r="AA3" s="12" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="AB3" s="12" t="inlineStr">
+        <is>
+          <t>AGH Corp US</t>
+        </is>
+      </c>
+      <c r="AC3" s="12" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AD3" s="12" t="inlineStr">
         <is>
           <t>Acme</t>
         </is>
       </c>
-      <c r="M3" s="12" t="inlineStr">
+      <c r="AE3" s="12" t="inlineStr">
         <is>
           <t>Global</t>
         </is>
       </c>
-      <c r="N3" s="12" t="inlineStr">
-        <is>
-          <t>Holdings</t>
-        </is>
-      </c>
-      <c r="O3" s="12" t="inlineStr">
+      <c r="AF3" s="12" t="inlineStr">
+        <is>
+          <t>LLC</t>
+        </is>
+      </c>
+      <c r="AG3" s="12" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="P3" s="12" t="inlineStr">
-        <is>
-          <t>Acme Global Holdings LLC</t>
-        </is>
-      </c>
-      <c r="Q3" s="12" t="inlineStr">
+      <c r="AH3" s="12" t="inlineStr">
+        <is>
+          <t>Acme Global LLC</t>
+        </is>
+      </c>
+      <c r="AI3" s="12" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
       </c>
-      <c r="R3" s="12" t="inlineStr">
-        <is>
-          <t>Acme</t>
-        </is>
-      </c>
-      <c r="S3" s="12" t="inlineStr">
-        <is>
-          <t>Intl</t>
-        </is>
-      </c>
-      <c r="T3" s="12" t="inlineStr">
-        <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="U3" s="12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="V3" s="12" t="inlineStr">
-        <is>
-          <t>Acme International Group</t>
-        </is>
-      </c>
-      <c r="W3" s="12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="X3" s="12" t="inlineStr">
-        <is>
-          <t>AGH</t>
-        </is>
-      </c>
-      <c r="Y3" s="12" t="inlineStr">
-        <is>
-          <t>Corp</t>
-        </is>
-      </c>
-      <c r="Z3" s="12" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="AA3" s="12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AB3" s="12" t="inlineStr">
-        <is>
-          <t>AGH Corp US</t>
-        </is>
-      </c>
-      <c r="AC3" s="12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AD3" s="12" t="inlineStr">
-        <is>
-          <t>Acme</t>
-        </is>
-      </c>
-      <c r="AE3" s="12" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
-      <c r="AF3" s="12" t="inlineStr">
-        <is>
-          <t>LLC</t>
-        </is>
-      </c>
-      <c r="AG3" s="12" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="AH3" s="12" t="inlineStr">
-        <is>
-          <t>Acme Global LLC</t>
-        </is>
-      </c>
-      <c r="AI3" s="12" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
       <c r="AJ3" s="12" t="inlineStr">
         <is>
           <t>500 Market Street</t>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="AN3" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="AO3" s="12" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="AT3" s="12" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>GBR</t>
         </is>
       </c>
       <c r="AU3" s="12" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="AZ3" s="12" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="BA3" s="12" t="inlineStr">
@@ -3116,7 +3116,7 @@
       </c>
       <c r="BD3" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="BE3" s="12" t="inlineStr">
@@ -3126,17 +3126,17 @@
       </c>
       <c r="BF3" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="BG3" s="12" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>GBR</t>
         </is>
       </c>
       <c r="BH3" s="12" t="inlineStr">
         <is>
-          <t>CA</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="BI3" s="12" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="E4" s="12" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="F4" s="12" t="inlineStr">
@@ -3188,7 +3188,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="I4" s="12" t="inlineStr">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="K4" s="12" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="L4" s="12" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="AN4" s="12" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="AO4" s="12" t="inlineStr">
@@ -3378,7 +3378,7 @@
       </c>
       <c r="AT4" s="12" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>ARE</t>
         </is>
       </c>
       <c r="AU4" s="12" t="inlineStr">
@@ -3408,14 +3408,14 @@
       </c>
       <c r="AZ4" s="12" t="inlineStr">
         <is>
+          <t>SGP</t>
+        </is>
+      </c>
+      <c r="BA4" s="12" t="inlineStr">
+        <is>
           <t>SG</t>
         </is>
       </c>
-      <c r="BA4" s="12" t="inlineStr">
-        <is>
-          <t>SG</t>
-        </is>
-      </c>
       <c r="BB4" s="12" t="inlineStr">
         <is>
           <t>1992-11-30</t>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="BD4" s="12" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="BE4" s="12" t="inlineStr">
@@ -3438,17 +3438,17 @@
       </c>
       <c r="BF4" s="12" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IND</t>
         </is>
       </c>
       <c r="BG4" s="12" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>ARE</t>
         </is>
       </c>
       <c r="BH4" s="12" t="inlineStr">
         <is>
-          <t>SG</t>
+          <t>SGP</t>
         </is>
       </c>
       <c r="BI4" s="12" t="inlineStr">

</xml_diff>